<commit_message>
pagina filha com codigos reinf e atualização de planilhas
</commit_message>
<xml_diff>
--- a/upload/f500.xlsx
+++ b/upload/f500.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/597695ca0a7eda65/Documentos/Inovare/Netsuite/layout de importação por planilha/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/597695ca0a7eda65/Documentos/Inovare/Netsuite/doc-netsuite/upload/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="40" documentId="8_{FF58B0EA-7845-4958-85FC-528124269E04}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B4A33C96-F38E-410D-AB45-17C4C05D8324}"/>
+  <xr:revisionPtr revIDLastSave="43" documentId="8_{FF58B0EA-7845-4958-85FC-528124269E04}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4E28B507-B4FA-4EA2-95BC-B3C19C3E7253}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{7917F040-528D-4EE8-B827-0BC031F7DA00}"/>
   </bookViews>
@@ -71,7 +71,7 @@
         <t>[Comentário encadeado]
 Sua versão do Excel permite que você leia este comentário encadeado, no entanto, as edições serão removidas se o arquivo for aberto em uma versão mais recente do Excel. Saiba mais: https://go.microsoft.com/fwlink/?linkid=870924
 Comentário:
-    Data em que o registro deve ser escriturado</t>
+    Data em que o registro deve ser escriturado no formato: DD/MM/AAAA. Exemplo: 31/10/2023.</t>
       </text>
     </comment>
     <comment ref="C1" authorId="2" shapeId="0" xr:uid="{2F9F7CEA-5D5C-468A-A2F4-9A47AFF5EE95}">
@@ -319,13 +319,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -670,7 +672,7 @@
     <text>CNPJ da empresa onde o registro deve ser escriturado</text>
   </threadedComment>
   <threadedComment ref="B1" dT="2025-09-22T19:33:14.26" personId="{4991DAD8-94C7-491C-A72C-1C75F7BED0C8}" id="{B8D67E0C-A8A5-4FA1-8077-77CFCCAC7FAA}">
-    <text>Data em que o registro deve ser escriturado</text>
+    <text>Data em que o registro deve ser escriturado no formato: DD/MM/AAAA. Exemplo: 31/10/2023.</text>
   </threadedComment>
   <threadedComment ref="C1" dT="2025-09-22T19:33:26.70" personId="{4991DAD8-94C7-491C-A72C-1C75F7BED0C8}" id="{2F9F7CEA-5D5C-468A-A2F4-9A47AFF5EE95}">
     <text>CST de PIS</text>
@@ -729,7 +731,7 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15.109375" style="3" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.33203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.33203125" style="7" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="8.44140625" style="3" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="6.77734375" style="5" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="11.109375" style="3" bestFit="1" customWidth="1"/>
@@ -752,7 +754,7 @@
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="6" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="2" t="s">
@@ -808,7 +810,7 @@
       <c r="A2" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="7" t="s">
         <v>20</v>
       </c>
       <c r="C2" s="3" t="s">

</xml_diff>